<commit_message>
feat: add BEJ48 19th generation birthdays
</commit_message>
<xml_diff>
--- a/SNH48成员名单生日表2603 (1).xlsx
+++ b/SNH48成员名单生日表2603 (1).xlsx
@@ -898,7 +898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1053"/>
+  <dimension ref="A1:H1061"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="3" min="1" max="1"/>
@@ -29554,7 +29554,7 @@
       </c>
       <c r="H1052" s="3" t="n"/>
     </row>
-    <row r="1053">
+    <row r="1053" s="12">
       <c r="A1053" s="3" t="n">
         <v>81</v>
       </c>
@@ -29581,6 +29581,230 @@
         <v>357</v>
       </c>
       <c r="H1053" s="3" t="n"/>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1054" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1054" s="3" t="inlineStr">
+        <is>
+          <t>范小天</t>
+        </is>
+      </c>
+      <c r="D1054" s="6" t="n">
+        <v>38369</v>
+      </c>
+      <c r="E1054" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1054" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1054" s="0" t="n">
+        <v>252</v>
+      </c>
+      <c r="H1054" s="3" t="n"/>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1055" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1055" s="3" t="inlineStr">
+        <is>
+          <t>刘雨硕</t>
+        </is>
+      </c>
+      <c r="D1055" s="6" t="n">
+        <v>38566</v>
+      </c>
+      <c r="E1055" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1055" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1055" s="0" t="n">
+        <v>55</v>
+      </c>
+      <c r="H1055" s="3" t="n"/>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1056" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1056" s="3" t="inlineStr">
+        <is>
+          <t>刘卓尔</t>
+        </is>
+      </c>
+      <c r="D1056" s="6" t="n">
+        <v>38128</v>
+      </c>
+      <c r="E1056" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1056" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="G1056" s="0" t="n">
+        <v>128</v>
+      </c>
+      <c r="H1056" s="3" t="n"/>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1057" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1057" s="3" t="inlineStr">
+        <is>
+          <t>李祉瑶</t>
+        </is>
+      </c>
+      <c r="D1057" s="6" t="n">
+        <v>39957</v>
+      </c>
+      <c r="E1057" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1057" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1057" s="0" t="n">
+        <v>125</v>
+      </c>
+      <c r="H1057" s="3" t="n"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1058" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1058" s="3" t="inlineStr">
+        <is>
+          <t>武佳凝</t>
+        </is>
+      </c>
+      <c r="D1058" s="6" t="n">
+        <v>40046</v>
+      </c>
+      <c r="E1058" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1058" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1058" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1058" s="3" t="n"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1059" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1059" s="3" t="inlineStr">
+        <is>
+          <t>王馨怡</t>
+        </is>
+      </c>
+      <c r="D1059" s="6" t="n">
+        <v>39839</v>
+      </c>
+      <c r="E1059" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1059" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1059" s="0" t="n">
+        <v>243</v>
+      </c>
+      <c r="H1059" s="3" t="n"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1060" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1060" s="3" t="inlineStr">
+        <is>
+          <t>张旭</t>
+        </is>
+      </c>
+      <c r="D1060" s="6" t="n">
+        <v>39200</v>
+      </c>
+      <c r="E1060" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1060" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="G1060" s="0" t="n">
+        <v>151</v>
+      </c>
+      <c r="H1060" s="3" t="n"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="B1061" s="2" t="inlineStr">
+        <is>
+          <t>BEJ48十九期生</t>
+        </is>
+      </c>
+      <c r="C1061" s="3" t="inlineStr">
+        <is>
+          <t>张怡璐</t>
+        </is>
+      </c>
+      <c r="D1061" s="6" t="n">
+        <v>38293</v>
+      </c>
+      <c r="E1061" s="6" t="n">
+        <v>46291</v>
+      </c>
+      <c r="F1061" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1061" s="0" t="n">
+        <v>328</v>
+      </c>
+      <c r="H1061" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>